<commit_message>
Add docker-compose config, update data files with restaurant invoice test
</commit_message>
<xml_diff>
--- a/extracted_invoices.xlsx
+++ b/extracted_invoices.xlsx
@@ -431,13 +431,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
@@ -605,6 +605,49 @@
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>INV-2024-215</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02/08/2024</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>16/08/2024</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ravi Restaurant Supplies</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>27RAVIX9988K1Z7</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>12400.00</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Stainless Steel Tiffin Boxes (qty: 30, price: 180.00, total: 5400.00) | Commercial Gas Burner (qty: 2, price: 3500.00, total: 7000.00)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>